<commit_message>
Please provide the file changes or a description of the code modifications so I can generate the commit message for you.
</commit_message>
<xml_diff>
--- a/OI/jeu_du_kanban/clé USB Jeu du Kanban/Tableau de bord 25032026.xlsx
+++ b/OI/jeu_du_kanban/clé USB Jeu du Kanban/Tableau de bord 25032026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/jeu_du_kanban/clé USB Jeu du Kanban/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{7A3549F7-05CD-498B-87C6-4795445A1221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54AEBAC8-DFD8-44BC-AA32-65C69CE7CF5A}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{7A3549F7-05CD-498B-87C6-4795445A1221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E405A5A2-8665-4346-868F-726FED7F0579}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="17472" windowHeight="10992" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Graphique" sheetId="36" r:id="rId1"/>
@@ -479,6 +479,15 @@
               <c:numCache>
                 <c:formatCode>"€"#,##0_);\("€"#,##0\)</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2055</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1555</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1700</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -540,6 +549,15 @@
               <c:numCache>
                 <c:formatCode>"€"#,##0_);\("€"#,##0\)</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2259</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1162</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1546</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -601,6 +619,15 @@
               <c:numCache>
                 <c:formatCode>"€"#,##0_);\("€"#,##0\)</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1945</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>725</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1554</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -864,6 +891,15 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.91500000000000004</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.98499999999999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.94</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -925,6 +961,15 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.95</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.62</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.06</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -986,6 +1031,15 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.89</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.81</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.82</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1067,7 +1121,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
-          <c:min val="0.30000000000000004"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1249,6 +1303,15 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.73</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.74199999999999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.75</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1310,6 +1373,15 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.63</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.72</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.7</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -1371,6 +1443,15 @@
               <c:numCache>
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.67</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.72199999999999998</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.8</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -2432,14 +2513,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="9" width="14.28515625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="13.7109375" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="9" width="14.27734375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="13.71875" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="23" t="s">
         <v>10</v>
       </c>
@@ -2456,7 +2537,7 @@
       <c r="H1" s="24"/>
       <c r="I1" s="25"/>
     </row>
-    <row r="2" spans="1:9" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="5.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="3"/>
       <c r="B2" s="2"/>
       <c r="C2" s="4"/>
@@ -2467,7 +2548,7 @@
       <c r="H2" s="2"/>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="3"/>
       <c r="B3" s="2"/>
       <c r="C3" s="4"/>
@@ -2478,7 +2559,7 @@
       <c r="H3" s="2"/>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="3"/>
       <c r="B4" s="2"/>
       <c r="C4" s="4"/>
@@ -2489,7 +2570,7 @@
       <c r="H4" s="2"/>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="3"/>
       <c r="B5" s="2"/>
       <c r="C5" s="4"/>
@@ -2500,7 +2581,7 @@
       <c r="H5" s="2"/>
       <c r="I5" s="4"/>
     </row>
-    <row r="6" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="3"/>
       <c r="B6" s="2"/>
       <c r="C6" s="4"/>
@@ -2511,7 +2592,7 @@
       <c r="H6" s="2"/>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="3"/>
       <c r="B7" s="2"/>
       <c r="C7" s="4"/>
@@ -2522,7 +2603,7 @@
       <c r="H7" s="2"/>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="3"/>
       <c r="B8" s="2"/>
       <c r="C8" s="4"/>
@@ -2533,7 +2614,7 @@
       <c r="H8" s="2"/>
       <c r="I8" s="4"/>
     </row>
-    <row r="9" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="3"/>
       <c r="B9" s="2"/>
       <c r="C9" s="4"/>
@@ -2544,7 +2625,7 @@
       <c r="H9" s="2"/>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="3"/>
       <c r="B10" s="2"/>
       <c r="C10" s="4"/>
@@ -2555,7 +2636,7 @@
       <c r="H10" s="2"/>
       <c r="I10" s="4"/>
     </row>
-    <row r="11" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="3"/>
       <c r="B11" s="2"/>
       <c r="C11" s="4"/>
@@ -2566,7 +2647,7 @@
       <c r="H11" s="2"/>
       <c r="I11" s="4"/>
     </row>
-    <row r="12" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="3"/>
       <c r="B12" s="2"/>
       <c r="C12" s="4"/>
@@ -2577,7 +2658,7 @@
       <c r="H12" s="2"/>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="3"/>
       <c r="B13" s="2"/>
       <c r="C13" s="4"/>
@@ -2588,7 +2669,7 @@
       <c r="H13" s="2"/>
       <c r="I13" s="4"/>
     </row>
-    <row r="14" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="3"/>
       <c r="B14" s="2"/>
       <c r="C14" s="4"/>
@@ -2599,7 +2680,7 @@
       <c r="H14" s="2"/>
       <c r="I14" s="4"/>
     </row>
-    <row r="15" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="3"/>
       <c r="B15" s="2"/>
       <c r="C15" s="4"/>
@@ -2610,7 +2691,7 @@
       <c r="H15" s="2"/>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="3"/>
       <c r="B16" s="2"/>
       <c r="C16" s="4"/>
@@ -2621,7 +2702,7 @@
       <c r="H16" s="2"/>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="3"/>
       <c r="B17" s="2"/>
       <c r="C17" s="4"/>
@@ -2632,7 +2713,7 @@
       <c r="H17" s="2"/>
       <c r="I17" s="4"/>
     </row>
-    <row r="18" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="5"/>
       <c r="B18" s="6"/>
       <c r="C18" s="7"/>
@@ -2643,7 +2724,7 @@
       <c r="H18" s="6"/>
       <c r="I18" s="7"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -2654,7 +2735,7 @@
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A23" s="22" t="s">
         <v>15</v>
       </c>
@@ -2676,14 +2757,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:E16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="27.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="27.5546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
@@ -2700,35 +2781,50 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-    </row>
-    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="10">
+        <v>0.91500000000000004</v>
+      </c>
+      <c r="C3" s="10">
+        <v>0.98499999999999999</v>
+      </c>
+      <c r="E3" s="10">
+        <v>0.94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-    </row>
-    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="12">
+        <v>0.95</v>
+      </c>
+      <c r="C4" s="12">
+        <v>0.62</v>
+      </c>
+      <c r="E4" s="12">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-    </row>
-    <row r="6" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="7" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="14">
+        <v>0.89</v>
+      </c>
+      <c r="C5" s="14">
+        <v>0.81</v>
+      </c>
+      <c r="E5" s="14">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="7" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="8" t="s">
         <v>14</v>
       </c>
@@ -2745,35 +2841,50 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-    </row>
-    <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="10">
+        <v>0.73</v>
+      </c>
+      <c r="C8" s="10">
+        <v>0.74199999999999999</v>
+      </c>
+      <c r="E8" s="10">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-    </row>
-    <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="12">
+        <v>0.63</v>
+      </c>
+      <c r="C9" s="12">
+        <v>0.72</v>
+      </c>
+      <c r="E9" s="12">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-    </row>
-    <row r="11" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="12" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="14">
+        <v>0.67</v>
+      </c>
+      <c r="C10" s="14">
+        <v>0.72199999999999998</v>
+      </c>
+      <c r="E10" s="14">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="12" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B12" s="15" t="s">
         <v>2</v>
       </c>
@@ -2787,7 +2898,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="8" t="s">
         <v>1</v>
       </c>
@@ -2804,32 +2915,50 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="16"/>
-      <c r="C14" s="17"/>
+      <c r="B14" s="16">
+        <v>2055</v>
+      </c>
+      <c r="C14" s="17">
+        <v>1555</v>
+      </c>
       <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-    </row>
-    <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E14" s="17">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="19"/>
+      <c r="B15" s="18">
+        <v>2259</v>
+      </c>
+      <c r="C15" s="19">
+        <v>1162</v>
+      </c>
       <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-    </row>
-    <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E15" s="19">
+        <v>1546</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="20"/>
-      <c r="C16" s="21"/>
+      <c r="B16" s="20">
+        <v>1945</v>
+      </c>
+      <c r="C16" s="21">
+        <v>725</v>
+      </c>
       <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
+      <c r="E16" s="21">
+        <v>1554</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="0" type="noConversion"/>

</xml_diff>